<commit_message>
R6 - ri_design_properties.xlsx round-trip, no net change
membrane_factor was added then retracted the same session: Eq 3-26's
membrane factor Ω turned out to belong on GeosyntheticLayerDesign as a plain
scalar (diggs-schema), not a dictionary-bound AuthorizedParameter, so no
entry was needed after all. The regenerated XML is byte-identical to
baseline; only this workbook's binary round-trips (openpyxl save artifact,
cell content unchanged - 14 entries before and after).
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/ri_design_properties.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/ri_design_properties.xlsx
@@ -1010,7 +1010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="7" customWidth="1" style="2" min="1" max="1"/>
@@ -1572,7 +1572,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2">
-        <f>IF(ISNA(VLOOKUP(B19,AssociatedElements!B$2:B2957,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B20,AssociatedElements!B$2:B2958,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B16" s="13" t="n"/>
@@ -1584,7 +1584,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2">
-        <f>IF(ISNA(VLOOKUP(B20,AssociatedElements!B$2:B2958,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B21,AssociatedElements!B$2:B2959,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B17" s="13" t="n"/>
@@ -1596,7 +1596,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2">
-        <f>IF(ISNA(VLOOKUP(B21,AssociatedElements!B$2:B2959,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B22,AssociatedElements!B$2:B2960,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B18" s="13" t="n"/>
@@ -1608,7 +1608,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2">
-        <f>IF(ISNA(VLOOKUP(B22,AssociatedElements!B$2:B2960,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B23,AssociatedElements!B$2:B2961,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B19" s="13" t="n"/>
@@ -1620,27 +1620,26 @@
     </row>
     <row r="20">
       <c r="A20" s="2">
-        <f>IF(ISNA(VLOOKUP(B23,AssociatedElements!B$2:B2961,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B20" s="13" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B24,AssociatedElements!B$2:B2962,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="D20" s="16" t="n"/>
       <c r="G20" s="9" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2">
-        <f>IF(ISNA(VLOOKUP(B24,AssociatedElements!B$2:B2962,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="D21" s="16" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B25,AssociatedElements!B$2:B2963,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="E21" s="13" t="n"/>
+      <c r="F21" s="13" t="n"/>
       <c r="G21" s="9" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2">
-        <f>IF(ISNA(VLOOKUP(B25,AssociatedElements!B$2:B2963,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B26,AssociatedElements!B$2:B2964,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B22" s="13" t="n"/>
@@ -1651,30 +1650,31 @@
     </row>
     <row r="23">
       <c r="A23" s="2">
-        <f>IF(ISNA(VLOOKUP(B26,AssociatedElements!B$2:B2964,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B27,AssociatedElements!B$2:B2965,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B23" s="13" t="n"/>
       <c r="C23" s="13" t="n"/>
+      <c r="D23" s="15" t="n"/>
       <c r="E23" s="13" t="n"/>
       <c r="F23" s="13" t="n"/>
       <c r="G23" s="9" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2">
-        <f>IF(ISNA(VLOOKUP(B27,AssociatedElements!B$2:B2965,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B28,AssociatedElements!B$2:B2966,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B24" s="13" t="n"/>
       <c r="C24" s="13" t="n"/>
-      <c r="D24" s="15" t="n"/>
+      <c r="D24" s="14" t="n"/>
       <c r="E24" s="13" t="n"/>
       <c r="F24" s="13" t="n"/>
       <c r="G24" s="9" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2">
-        <f>IF(ISNA(VLOOKUP(B28,AssociatedElements!B$2:B2966,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B29,AssociatedElements!B$2:B2967,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B25" s="13" t="n"/>
@@ -1686,7 +1686,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2">
-        <f>IF(ISNA(VLOOKUP(B29,AssociatedElements!B$2:B2967,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B30,AssociatedElements!B$2:B2968,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B26" s="13" t="n"/>
@@ -1698,19 +1698,19 @@
     </row>
     <row r="27">
       <c r="A27" s="2">
-        <f>IF(ISNA(VLOOKUP(B30,AssociatedElements!B$2:B2968,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B31,AssociatedElements!B$2:B2969,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B27" s="13" t="n"/>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="14" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
+      <c r="C27" s="18" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="18" t="n"/>
+      <c r="F27" s="18" t="n"/>
       <c r="G27" s="9" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2">
-        <f>IF(ISNA(VLOOKUP(B31,AssociatedElements!B$2:B2969,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B32,AssociatedElements!B$2:B2970,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B28" s="13" t="n"/>
@@ -1722,7 +1722,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2">
-        <f>IF(ISNA(VLOOKUP(B32,AssociatedElements!B$2:B2970,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B33,AssociatedElements!B$2:B2971,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B29" s="13" t="n"/>
@@ -1734,7 +1734,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2">
-        <f>IF(ISNA(VLOOKUP(B33,AssociatedElements!B$2:B2971,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B34,AssociatedElements!B$2:B2972,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B30" s="13" t="n"/>
@@ -1746,7 +1746,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2">
-        <f>IF(ISNA(VLOOKUP(B34,AssociatedElements!B$2:B2972,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B35,AssociatedElements!B$2:B2973,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B31" s="13" t="n"/>
@@ -1758,7 +1758,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2">
-        <f>IF(ISNA(VLOOKUP(B35,AssociatedElements!B$2:B2973,1,FALSE)),"Not used","")</f>
+        <f>IF(ISNA(VLOOKUP(B36,AssociatedElements!B$2:B2974,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
       <c r="B32" s="13" t="n"/>
@@ -1770,22 +1770,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2">
-        <f>IF(ISNA(VLOOKUP(B36,AssociatedElements!B$2:B2974,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B33" s="13" t="n"/>
-      <c r="C33" s="18" t="n"/>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="18" t="n"/>
-      <c r="F33" s="18" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B37,AssociatedElements!B$2:B2975,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
       <c r="G33" s="9" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2">
-        <f>IF(ISNA(VLOOKUP(B37,AssociatedElements!B$2:B2975,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="G34" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1802,7 +1790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="6.83203125" customWidth="1" min="1" max="1"/>
@@ -2129,136 +2117,129 @@
     </row>
     <row r="16">
       <c r="A16">
-        <f>IF(ISNA(VLOOKUP(B19,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B20,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B16" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="A17">
-        <f>IF(ISNA(VLOOKUP(B20,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B21,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B17" s="20" t="n"/>
     </row>
     <row r="18">
       <c r="A18">
-        <f>IF(ISNA(VLOOKUP(B21,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B18" s="20" t="n"/>
     </row>
     <row r="19">
       <c r="A19">
-        <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B19" s="20" t="n"/>
     </row>
     <row r="20">
       <c r="A20">
-        <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B20" s="20" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21">
-        <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22">
-        <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B26,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23">
-        <f>IF(ISNA(VLOOKUP(B26,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B23" s="2" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B23" s="13" t="n"/>
     </row>
     <row r="24">
       <c r="A24">
-        <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B28,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="A25">
-        <f>IF(ISNA(VLOOKUP(B28,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B29,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26">
-        <f>IF(ISNA(VLOOKUP(B29,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B30,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B26" s="13" t="n"/>
     </row>
     <row r="27">
       <c r="A27">
-        <f>IF(ISNA(VLOOKUP(B30,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28">
-        <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B32,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B28" s="13" t="n"/>
     </row>
     <row r="29">
       <c r="A29">
-        <f>IF(ISNA(VLOOKUP(B32,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B33,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B29" s="13" t="n"/>
     </row>
     <row r="30">
       <c r="A30">
-        <f>IF(ISNA(VLOOKUP(B33,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B34,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B30" s="13" t="n"/>
     </row>
     <row r="31">
       <c r="A31">
-        <f>IF(ISNA(VLOOKUP(B34,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B35,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B31" s="13" t="n"/>
     </row>
     <row r="32">
       <c r="A32">
-        <f>IF(ISNA(VLOOKUP(B35,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <f>IF(ISNA(VLOOKUP(B36,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
       <c r="B32" s="13" t="n"/>
     </row>
     <row r="33">
       <c r="A33">
-        <f>IF(ISNA(VLOOKUP(B36,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B33" s="13" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34">
         <f>IF(ISNA(VLOOKUP(B37,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B34" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>